<commit_message>
feat: agregado scraper y vis plano
</commit_message>
<xml_diff>
--- a/backend/docs/VIS-PLA.xlsx
+++ b/backend/docs/VIS-PLA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\planos-react-app\backend\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2278BDD2-46F2-44FE-BB06-5A1B94CE209A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2410EC58-5F3C-4D31-A405-E11A654ED0AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A2F3C56B-C265-481F-806E-CD3616F017BF}"/>
   </bookViews>
@@ -212,9 +212,6 @@
     <t>B.25 Trámite municipal</t>
   </si>
   <si>
-    <t>B.11 Subsanacion de observaciones SUNARP (si fuera el caso)</t>
-  </si>
-  <si>
     <t>B.12 FUE (Formulario Unico de Edifcaciones)</t>
   </si>
   <si>
@@ -324,6 +321,9 @@
   </si>
   <si>
     <t>Av. Guillermo Billinghurst 1081, Oficina 202 - SJM</t>
+  </si>
+  <si>
+    <t>B.11 Subsanacion de observaciones Municipio (si fuera el caso)</t>
   </si>
 </sst>
 </file>
@@ -1927,9 +1927,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1967,7 +1967,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2073,7 +2073,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2215,7 +2215,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2248,7 +2248,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="46" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E4" s="46"/>
       <c r="F4" s="46"/>
@@ -2259,7 +2259,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="47" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E5" s="47"/>
       <c r="F5" s="47"/>
@@ -2270,7 +2270,7 @@
         <v>3</v>
       </c>
       <c r="D6" s="48" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E6" s="48"/>
       <c r="F6" s="48"/>
@@ -2281,7 +2281,7 @@
         <v>4</v>
       </c>
       <c r="D7" s="49" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E7" s="49"/>
       <c r="F7" s="49"/>
@@ -2355,7 +2355,7 @@
     </row>
     <row r="14" spans="1:8" s="11" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B14" s="44"/>
       <c r="C14" s="13" t="s">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="E17" s="19">
         <f ca="1">TODAY()</f>
-        <v>46163</v>
+        <v>46213</v>
       </c>
       <c r="F17" s="15"/>
       <c r="G17" s="15"/>
@@ -2736,11 +2736,11 @@
     </row>
     <row r="42" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="10"/>
-      <c r="B42" s="73" t="s">
-        <v>57</v>
-      </c>
-      <c r="C42" s="74"/>
-      <c r="D42" s="75"/>
+      <c r="B42" s="93" t="s">
+        <v>94</v>
+      </c>
+      <c r="C42" s="94"/>
+      <c r="D42" s="95"/>
       <c r="E42" s="79"/>
       <c r="F42" s="80"/>
       <c r="G42" s="81"/>
@@ -2749,12 +2749,12 @@
     <row r="43" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="10"/>
       <c r="B43" s="73" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C43" s="74"/>
       <c r="D43" s="75"/>
       <c r="E43" s="102" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F43" s="103"/>
       <c r="G43" s="104"/>
@@ -2763,7 +2763,7 @@
     <row r="44" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10"/>
       <c r="B44" s="93" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C44" s="94"/>
       <c r="D44" s="95"/>
@@ -2775,7 +2775,7 @@
     <row r="45" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10"/>
       <c r="B45" s="73" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C45" s="74"/>
       <c r="D45" s="75"/>
@@ -2786,7 +2786,7 @@
     </row>
     <row r="46" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="66" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C46" s="67"/>
       <c r="D46" s="67"/>
@@ -2798,12 +2798,12 @@
     <row r="47" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
       <c r="B47" s="128" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C47" s="129"/>
       <c r="D47" s="130"/>
       <c r="E47" s="51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F47" s="52"/>
       <c r="G47" s="53"/>
@@ -2815,7 +2815,7 @@
       <c r="C48" s="132"/>
       <c r="D48" s="133"/>
       <c r="E48" s="114" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F48" s="115"/>
       <c r="G48" s="116"/>
@@ -2827,7 +2827,7 @@
       <c r="C49" s="132"/>
       <c r="D49" s="133"/>
       <c r="E49" s="117" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F49" s="118"/>
       <c r="G49" s="119"/>
@@ -2836,7 +2836,7 @@
     <row r="50" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="10"/>
       <c r="B50" s="120" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C50" s="121"/>
       <c r="D50" s="122"/>
@@ -2858,7 +2858,7 @@
     <row r="52" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="10"/>
       <c r="B52" s="34" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C52" s="127"/>
       <c r="D52" s="127"/>
@@ -2900,7 +2900,7 @@
     <row r="56" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="21"/>
       <c r="B56" s="136" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C56" s="136"/>
       <c r="D56" s="136"/>
@@ -2912,14 +2912,14 @@
     <row r="57" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="22"/>
       <c r="B57" s="137" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C57" s="137"/>
       <c r="D57" s="35">
         <v>6</v>
       </c>
       <c r="E57" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F57" s="20"/>
       <c r="G57" s="20"/>
@@ -2928,7 +2928,7 @@
     <row r="58" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="21"/>
       <c r="B58" s="136" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C58" s="136"/>
       <c r="D58" s="136"/>
@@ -2940,7 +2940,7 @@
     <row r="59" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="22"/>
       <c r="B59" s="138" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C59" s="138"/>
       <c r="D59" s="37">
@@ -2948,7 +2948,7 @@
         <v>0</v>
       </c>
       <c r="E59" s="139" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F59" s="139"/>
       <c r="G59" s="20"/>
@@ -2957,7 +2957,7 @@
     <row r="60" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="21"/>
       <c r="B60" s="136" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C60" s="136"/>
       <c r="D60" s="136"/>
@@ -2969,43 +2969,43 @@
     <row r="61" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="22"/>
       <c r="B61" s="36" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C61" s="37"/>
       <c r="D61" s="140" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E61" s="141"/>
       <c r="F61" s="141"/>
       <c r="G61" s="38">
         <f ca="1">E17</f>
-        <v>46163</v>
+        <v>46213</v>
       </c>
       <c r="H61" s="22"/>
     </row>
     <row r="62" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="22"/>
       <c r="B62" s="36" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C62" s="39"/>
       <c r="D62" s="141" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E62" s="141"/>
       <c r="F62" s="141"/>
       <c r="G62" s="38">
         <f ca="1">E17+8</f>
-        <v>46171</v>
+        <v>46221</v>
       </c>
       <c r="H62" s="40" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="63" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="10"/>
       <c r="B63" s="142" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C63" s="142"/>
       <c r="D63" s="142"/>
@@ -3016,10 +3016,10 @@
     </row>
     <row r="64" spans="1:8" s="23" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="42" t="s">
+        <v>76</v>
+      </c>
+      <c r="B64" s="134" t="s">
         <v>77</v>
-      </c>
-      <c r="B64" s="134" t="s">
-        <v>78</v>
       </c>
       <c r="C64" s="134"/>
       <c r="D64" s="134"/>
@@ -3029,39 +3029,39 @@
     </row>
     <row r="65" spans="2:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="143" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C65" s="143"/>
       <c r="D65" s="143"/>
       <c r="E65" s="143"/>
       <c r="F65" s="143" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G65" s="143"/>
       <c r="H65" s="143"/>
     </row>
     <row r="66" spans="2:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="144" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C66" s="144"/>
       <c r="D66" s="144"/>
       <c r="E66" s="144"/>
       <c r="F66" s="143" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G66" s="143"/>
       <c r="H66" s="143"/>
     </row>
     <row r="67" spans="2:8" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="144" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C67" s="144"/>
       <c r="D67" s="144"/>
       <c r="E67" s="144"/>
       <c r="F67" s="143" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G67" s="143"/>
       <c r="H67" s="143"/>
@@ -3195,7 +3195,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.59055118110236227" right="0.59055118110236227" top="0.59055118110236227" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="92" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="91" orientation="portrait" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>